<commit_message>
GitHub Action: generate latest manifests
</commit_message>
<xml_diff>
--- a/current-excel-manifests/FileAnnotationTemplate.xlsx
+++ b/current-excel-manifests/FileAnnotationTemplate.xlsx
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="561">
   <si>
     <t>Component</t>
   </si>
@@ -984,628 +984,631 @@
     <t>json</t>
   </si>
   <si>
+    <t>Emory_Levey_300_CSF_FNIH</t>
+  </si>
+  <si>
+    <t>transcript quantification</t>
+  </si>
+  <si>
+    <t>label free mass spectrometry</t>
+  </si>
+  <si>
+    <t>locs</t>
+  </si>
+  <si>
     <t>EmoryDrosophilaTau</t>
   </si>
   <si>
-    <t>transcript quantification</t>
-  </si>
-  <si>
-    <t>label free mass spectrometry</t>
-  </si>
-  <si>
-    <t>locs</t>
+    <t>variancePartition</t>
+  </si>
+  <si>
+    <t>Laser Speckle Imaging</t>
+  </si>
+  <si>
+    <t>maf</t>
   </si>
   <si>
     <t>EpiGABA</t>
   </si>
   <si>
-    <t>variancePartition</t>
-  </si>
-  <si>
-    <t>Laser Speckle Imaging</t>
-  </si>
-  <si>
-    <t>maf</t>
+    <t>Variant calling</t>
+  </si>
+  <si>
+    <t>LC-MS</t>
+  </si>
+  <si>
+    <t>mat</t>
   </si>
   <si>
     <t>EpiMap</t>
   </si>
   <si>
-    <t>Variant calling</t>
-  </si>
-  <si>
-    <t>LC-MS</t>
-  </si>
-  <si>
-    <t>mat</t>
+    <t>visualization</t>
+  </si>
+  <si>
+    <t>LC-MSMS</t>
+  </si>
+  <si>
+    <t>md</t>
   </si>
   <si>
     <t>eQTLmetaAnalysis</t>
   </si>
   <si>
-    <t>visualization</t>
-  </si>
-  <si>
-    <t>LC-MSMS</t>
-  </si>
-  <si>
-    <t>md</t>
+    <t>LC-SRM</t>
+  </si>
+  <si>
+    <t>mov</t>
   </si>
   <si>
     <t>FreshMicro</t>
   </si>
   <si>
-    <t>LC-SRM</t>
-  </si>
-  <si>
-    <t>mov</t>
+    <t>Leiden Oxylipins</t>
+  </si>
+  <si>
+    <t>mp4</t>
   </si>
   <si>
     <t>HBI_scRNAseq</t>
   </si>
   <si>
-    <t>Leiden Oxylipins</t>
-  </si>
-  <si>
-    <t>mp4</t>
+    <t>lentiMPRA</t>
+  </si>
+  <si>
+    <t>msf</t>
   </si>
   <si>
     <t>HBTRC</t>
   </si>
   <si>
-    <t>lentiMPRA</t>
-  </si>
-  <si>
-    <t>msf</t>
+    <t>LFP</t>
+  </si>
+  <si>
+    <t>mtx</t>
   </si>
   <si>
     <t>HDAC1-cKOBrain</t>
   </si>
   <si>
-    <t>LFP</t>
-  </si>
-  <si>
-    <t>mtx</t>
+    <t>liquid chromatography-electrochemical detection</t>
+  </si>
+  <si>
+    <t>nirs</t>
   </si>
   <si>
     <t>HumanFC</t>
   </si>
   <si>
-    <t>liquid chromatography-electrochemical detection</t>
-  </si>
-  <si>
-    <t>nirs</t>
+    <t>lncrnaSeq</t>
+  </si>
+  <si>
+    <t>pdf</t>
   </si>
   <si>
     <t>IL10_APPmouse</t>
   </si>
   <si>
-    <t>lncrnaSeq</t>
-  </si>
-  <si>
-    <t>pdf</t>
+    <t>locomotor activation behavior</t>
+  </si>
+  <si>
+    <t>pdresult</t>
   </si>
   <si>
     <t>iNiAstshRNA</t>
   </si>
   <si>
-    <t>locomotor activation behavior</t>
-  </si>
-  <si>
-    <t>pdresult</t>
+    <t>long-read rnaSeq</t>
+  </si>
+  <si>
+    <t>pdstudy</t>
   </si>
   <si>
     <t>IntegrativePathwayAnalysis</t>
   </si>
   <si>
-    <t>long-read rnaSeq</t>
-  </si>
-  <si>
-    <t>pdstudy</t>
+    <t>LTP</t>
+  </si>
+  <si>
+    <t>pdview</t>
   </si>
   <si>
     <t>iPSC</t>
   </si>
   <si>
-    <t>LTP</t>
-  </si>
-  <si>
-    <t>pdview</t>
+    <t>m6A-rnaSeq</t>
+  </si>
+  <si>
+    <t>plink</t>
   </si>
   <si>
     <t>iPSC-HiC</t>
   </si>
   <si>
-    <t>m6A-rnaSeq</t>
-  </si>
-  <si>
-    <t>plink</t>
+    <t>MDMS-SL</t>
+  </si>
+  <si>
+    <t>png</t>
   </si>
   <si>
     <t>iPSCAstrocytes</t>
   </si>
   <si>
-    <t>MDMS-SL</t>
-  </si>
-  <si>
-    <t>png</t>
+    <t>memory behavior</t>
+  </si>
+  <si>
+    <t>powerpoint</t>
   </si>
   <si>
     <t>iPSCMicroglia</t>
   </si>
   <si>
-    <t>memory behavior</t>
-  </si>
-  <si>
-    <t>powerpoint</t>
+    <t>Metabolon</t>
+  </si>
+  <si>
+    <t>Python script</t>
   </si>
   <si>
     <t>ISB_Taner_CollagenDomain</t>
   </si>
   <si>
-    <t>Metabolon</t>
-  </si>
-  <si>
-    <t>Python script</t>
+    <t>methylationArray</t>
+  </si>
+  <si>
+    <t>pzfx</t>
   </si>
   <si>
     <t>ISB_Taner_Cxcl10</t>
   </si>
   <si>
-    <t>methylationArray</t>
-  </si>
-  <si>
-    <t>pzfx</t>
+    <t>MIB/MS</t>
+  </si>
+  <si>
+    <t>R script</t>
   </si>
   <si>
     <t>ISB_Taner_PTN_MDK</t>
   </si>
   <si>
-    <t>MIB/MS</t>
-  </si>
-  <si>
-    <t>R script</t>
+    <t>microRNAcounts</t>
   </si>
   <si>
     <t>ISB_Taner_sIL10r_sIL4r</t>
   </si>
   <si>
-    <t>microRNAcounts</t>
+    <t>mirnaArray</t>
+  </si>
+  <si>
+    <t>RCC</t>
   </si>
   <si>
     <t>ISB_Taner_TGFbeta</t>
   </si>
   <si>
-    <t>mirnaArray</t>
-  </si>
-  <si>
-    <t>RCC</t>
+    <t>mirnaSeq</t>
+  </si>
+  <si>
+    <t>RData</t>
   </si>
   <si>
     <t>Jax.IU.Pitt.Proteomics_Metabolomics_Pilot</t>
   </si>
   <si>
-    <t>mirnaSeq</t>
-  </si>
-  <si>
-    <t>RData</t>
+    <t>MRI</t>
+  </si>
+  <si>
+    <t>recal</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_APOE4.Trem2.R47H</t>
   </si>
   <si>
-    <t>MRI</t>
-  </si>
-  <si>
-    <t>recal</t>
+    <t>mRNAcounts</t>
+  </si>
+  <si>
+    <t>RLF</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_APP.PS1</t>
   </si>
   <si>
-    <t>mRNAcounts</t>
-  </si>
-  <si>
-    <t>RLF</t>
+    <t>mRNAseq</t>
+  </si>
+  <si>
+    <t>rmd</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_Levetiracetam-5XFAD</t>
   </si>
   <si>
-    <t>mRNAseq</t>
-  </si>
-  <si>
-    <t>rmd</t>
+    <t>MudPIT</t>
+  </si>
+  <si>
+    <t>saf</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_LOAD2.PrimaryScreen</t>
   </si>
   <si>
-    <t>MudPIT</t>
-  </si>
-  <si>
-    <t>saf</t>
+    <t>nextGenerationTargetedSequencing</t>
+  </si>
+  <si>
+    <t>sam</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_MicrobiomePilot</t>
   </si>
   <si>
-    <t>nextGenerationTargetedSequencing</t>
-  </si>
-  <si>
-    <t>sam</t>
+    <t>Nightingale NMR</t>
+  </si>
+  <si>
+    <t>sav</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_PrimaryScreen</t>
   </si>
   <si>
-    <t>Nightingale NMR</t>
-  </si>
-  <si>
-    <t>sav</t>
+    <t>NOMe-Seq</t>
+  </si>
+  <si>
+    <t>sdf</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_StrainValidation</t>
   </si>
   <si>
-    <t>NOMe-Seq</t>
-  </si>
-  <si>
-    <t>sdf</t>
+    <t>novelty response behavior</t>
+  </si>
+  <si>
+    <t>seg</t>
   </si>
   <si>
     <t>Jax.IU.Pitt_Verubecestat_5XFAD</t>
   </si>
   <si>
-    <t>novelty response behavior</t>
-  </si>
-  <si>
-    <t>seg</t>
+    <t>open field test</t>
+  </si>
+  <si>
+    <t>Sentrix descriptor file</t>
   </si>
   <si>
     <t>LBP</t>
   </si>
   <si>
-    <t>open field test</t>
-  </si>
-  <si>
-    <t>Sentrix descriptor file</t>
+    <t>oxBS-Seq</t>
+  </si>
+  <si>
+    <t>sf3</t>
   </si>
   <si>
     <t>LillyMicroglia</t>
   </si>
   <si>
-    <t>oxBS-Seq</t>
-  </si>
-  <si>
-    <t>sf3</t>
+    <t>pharmacodynamics</t>
+  </si>
+  <si>
+    <t>sif</t>
   </si>
   <si>
     <t>LLFS</t>
   </si>
   <si>
-    <t>pharmacodynamics</t>
-  </si>
-  <si>
-    <t>sif</t>
+    <t>pharmacokinetics</t>
+  </si>
+  <si>
+    <t>sqlite</t>
   </si>
   <si>
     <t>lncRNA Pilot</t>
   </si>
   <si>
-    <t>pharmacokinetics</t>
-  </si>
-  <si>
-    <t>sqlite</t>
+    <t>photograph</t>
+  </si>
+  <si>
+    <t>sra</t>
   </si>
   <si>
     <t>MARS WISCONSIN</t>
   </si>
   <si>
-    <t>photograph</t>
-  </si>
-  <si>
-    <t>sra</t>
+    <t>polymeraseChainReaction</t>
+  </si>
+  <si>
+    <t>svg</t>
   </si>
   <si>
     <t>MayoeGWAS</t>
   </si>
   <si>
-    <t>polymeraseChainReaction</t>
-  </si>
-  <si>
-    <t>svg</t>
+    <t>Positron Emission Tomography</t>
+  </si>
+  <si>
+    <t>svs</t>
   </si>
   <si>
     <t>MayoHippocampus</t>
   </si>
   <si>
-    <t>Positron Emission Tomography</t>
-  </si>
-  <si>
-    <t>svs</t>
+    <t>proximity extension assay</t>
+  </si>
+  <si>
+    <t>Synapse Table</t>
   </si>
   <si>
     <t>MayoLOADGWAS</t>
   </si>
   <si>
-    <t>proximity extension assay</t>
-  </si>
-  <si>
-    <t>Synapse Table</t>
+    <t>questionnaire</t>
+  </si>
+  <si>
+    <t>tab</t>
   </si>
   <si>
     <t>MayoPilotRNAseq</t>
   </si>
   <si>
-    <t>questionnaire</t>
-  </si>
-  <si>
-    <t>tab</t>
+    <t>Rader Lipidomics</t>
+  </si>
+  <si>
+    <t>tagAlign</t>
   </si>
   <si>
     <t>MayoRNAseq</t>
   </si>
   <si>
-    <t>Rader Lipidomics</t>
-  </si>
-  <si>
-    <t>tagAlign</t>
+    <t>Real Time PCR</t>
+  </si>
+  <si>
+    <t>tar</t>
   </si>
   <si>
     <t>MC-BrAD</t>
   </si>
   <si>
-    <t>Real Time PCR</t>
-  </si>
-  <si>
-    <t>tar</t>
+    <t>Ribo-Seq</t>
+  </si>
+  <si>
+    <t>tbi</t>
   </si>
   <si>
     <t>MC-CAA</t>
   </si>
   <si>
-    <t>Ribo-Seq</t>
-  </si>
-  <si>
-    <t>tbi</t>
+    <t>rnaArray</t>
+  </si>
+  <si>
+    <t>tif</t>
   </si>
   <si>
     <t>MC_snRNA</t>
   </si>
   <si>
-    <t>rnaArray</t>
-  </si>
-  <si>
-    <t>tif</t>
+    <t>rnaSeq</t>
+  </si>
+  <si>
+    <t>tranches</t>
   </si>
   <si>
     <t>mCITE-Seq</t>
   </si>
   <si>
-    <t>rnaSeq</t>
-  </si>
-  <si>
-    <t>tranches</t>
+    <t>rotarod performance test</t>
+  </si>
+  <si>
+    <t>tsv</t>
   </si>
   <si>
     <t>MCMPS</t>
   </si>
   <si>
-    <t>rotarod performance test</t>
-  </si>
-  <si>
-    <t>tsv</t>
+    <t>RPPA</t>
+  </si>
+  <si>
+    <t>txt</t>
   </si>
   <si>
     <t>MEF2_Resilience</t>
   </si>
   <si>
-    <t>RPPA</t>
-  </si>
-  <si>
-    <t>txt</t>
+    <t>RRBS</t>
+  </si>
+  <si>
+    <t>vcf</t>
   </si>
   <si>
     <t>MindPhenomeKB</t>
   </si>
   <si>
-    <t>RRBS</t>
-  </si>
-  <si>
-    <t>vcf</t>
+    <t>sandwich ELISA</t>
+  </si>
+  <si>
+    <t>wiggle</t>
   </si>
   <si>
     <t>miR155</t>
   </si>
   <si>
-    <t>sandwich ELISA</t>
-  </si>
-  <si>
-    <t>wiggle</t>
+    <t>Sanger sequencing</t>
+  </si>
+  <si>
+    <t>xml</t>
   </si>
   <si>
     <t>MIT_ROSMAP_Multiomics</t>
   </si>
   <si>
-    <t>Sanger sequencing</t>
-  </si>
-  <si>
-    <t>xml</t>
+    <t>scale</t>
+  </si>
+  <si>
+    <t>yaml</t>
   </si>
   <si>
     <t>MOA-PAD</t>
   </si>
   <si>
-    <t>scale</t>
-  </si>
-  <si>
-    <t>yaml</t>
+    <t>scATACSeq</t>
+  </si>
+  <si>
+    <t>zip</t>
   </si>
   <si>
     <t>MODEL-AD_5XFAD</t>
   </si>
   <si>
-    <t>scATACSeq</t>
-  </si>
-  <si>
-    <t>zip</t>
+    <t>scCGIseq</t>
   </si>
   <si>
     <t>MODEL-AD_Abca7_APOE4_Trem2</t>
   </si>
   <si>
-    <t>scCGIseq</t>
+    <t>scirnaSeq</t>
   </si>
   <si>
     <t>MODEL-AD_APOE4_KI</t>
   </si>
   <si>
-    <t>scirnaSeq</t>
+    <t>scrnaSeq</t>
   </si>
   <si>
     <t>MODEL-AD_APOE4_Trem2</t>
   </si>
   <si>
-    <t>scrnaSeq</t>
+    <t>scwholeGenomeSeq</t>
   </si>
   <si>
     <t>MODEL-AD_Ceacam_KO_APOE4_Trem2</t>
   </si>
   <si>
-    <t>scwholeGenomeSeq</t>
+    <t>SiMoA</t>
   </si>
   <si>
     <t>MODEL-AD_hAbeta_KI</t>
   </si>
   <si>
-    <t>SiMoA</t>
+    <t>snATACSeq</t>
   </si>
   <si>
     <t>MODEL-AD_Harmonization</t>
   </si>
   <si>
-    <t>snATACSeq</t>
+    <t>snpArray</t>
   </si>
   <si>
     <t>MODEL-AD_hCR1_KI_on_APOE4_Trem2</t>
   </si>
   <si>
-    <t>snpArray</t>
+    <t>snrnaSeq</t>
   </si>
   <si>
     <t>MODEL-AD_hTau_Trem2</t>
   </si>
   <si>
-    <t>snrnaSeq</t>
+    <t>spontaneous alternation</t>
   </si>
   <si>
     <t>MODEL-AD_Il1rapKO_APOE4_Trem2_exon2KO</t>
   </si>
   <si>
-    <t>spontaneous alternation</t>
+    <t>STARRSeq</t>
   </si>
   <si>
     <t>MODEL-AD_Mthfr_APOE4_Trem2</t>
   </si>
   <si>
-    <t>STARRSeq</t>
+    <t>TMT quantitation</t>
   </si>
   <si>
     <t>MODEL-AD_Rat_F344</t>
   </si>
   <si>
-    <t>TMT quantitation</t>
+    <t>TotalRNAseq</t>
   </si>
   <si>
     <t>MODEL-AD_Trem2_R47H</t>
   </si>
   <si>
-    <t>TotalRNAseq</t>
+    <t>tractionForceMicroscopy</t>
   </si>
   <si>
     <t>MouseHAL</t>
   </si>
   <si>
-    <t>tractionForceMicroscopy</t>
+    <t>UC Davis GCTOF</t>
   </si>
   <si>
     <t>MRGWAS</t>
   </si>
   <si>
-    <t>UC Davis GCTOF</t>
+    <t>UCSD Untargeted Metabolomics</t>
   </si>
   <si>
     <t>MSBB</t>
   </si>
   <si>
-    <t>UCSD Untargeted Metabolomics</t>
+    <t>UPLC-ESI-QTOF-MS</t>
   </si>
   <si>
     <t>MSBB_ArrayTissuePanel</t>
   </si>
   <si>
-    <t>UPLC-ESI-QTOF-MS</t>
+    <t>UPLC-MSMS</t>
   </si>
   <si>
     <t>MSDM</t>
   </si>
   <si>
-    <t>UPLC-MSMS</t>
+    <t>Vernier Caliper</t>
   </si>
   <si>
     <t>MSMM</t>
   </si>
   <si>
-    <t>Vernier Caliper</t>
+    <t>von Frey test</t>
   </si>
   <si>
     <t>MSSMiPSC</t>
   </si>
   <si>
-    <t>von Frey test</t>
+    <t>westernBlot</t>
   </si>
   <si>
     <t>mtDNA_AD</t>
   </si>
   <si>
-    <t>westernBlot</t>
+    <t>wheel running</t>
   </si>
   <si>
     <t>NAPS</t>
   </si>
   <si>
-    <t>wheel running</t>
+    <t>whole-cell patch clamp</t>
   </si>
   <si>
     <t>NHP-Chimpanzee</t>
   </si>
   <si>
-    <t>whole-cell patch clamp</t>
+    <t>wholeGenomeSeq</t>
   </si>
   <si>
     <t>NHP-Macaque</t>
   </si>
   <si>
-    <t>wholeGenomeSeq</t>
+    <t>Wishart Catecholamines</t>
   </si>
   <si>
     <t>NPS-AD</t>
   </si>
   <si>
-    <t>Wishart Catecholamines</t>
+    <t>Wishart High Value Metabolites</t>
   </si>
   <si>
     <t>OFMM</t>
   </si>
   <si>
-    <t>Wishart High Value Metabolites</t>
+    <t>Zeno Electronic Walkway</t>
   </si>
   <si>
     <t>omicsADDS</t>
-  </si>
-  <si>
-    <t>Zeno Electronic Walkway</t>
   </si>
   <si>
     <t>Organoid_scRNAseq</t>
@@ -29184,37 +29187,40 @@
       <formula>$M1 = "metadata"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="O1:O1000">
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+      <formula>$K1 = "analysis"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N1:N1000">
+    <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
+      <formula>$K1 = "metadata"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L1:L1000">
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
+      <formula>$K1 = "experimentalData"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R1:R1000">
+    <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
       <formula>$K1 = "experimentalData"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F1000">
-    <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
-      <formula>$K1 = "experimentalData"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R1:R1000">
-    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
       <formula>$K1 = "experimentalData"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:M1000">
-    <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="7" stopIfTrue="1">
       <formula>$K1 = "experimentalData"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N1:N1000">
-    <cfRule type="expression" dxfId="0" priority="6" stopIfTrue="1">
-      <formula>$K1 = "metadata"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O1:O1000">
-    <cfRule type="expression" dxfId="0" priority="7" stopIfTrue="1">
-      <formula>$K1 = "analysis"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose one from dropdown" sqref="I2:I1000">
+      <formula1>Sheet2!$I$2:$I$185</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose one from dropdown" sqref="P2:P1000">
       <formula1>Sheet2!$P$2:$P$3</formula1>
     </dataValidation>
@@ -29226,9 +29232,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose one from dropdown" sqref="G2:G1000">
       <formula1>Sheet2!$G$2:$G$97</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose one from dropdown" sqref="I2:I1000">
-      <formula1>Sheet2!$I$2:$I$184</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Choose one from dropdown" sqref="Q2:Q1000">
       <formula1>Sheet2!$Q$2:$Q$26</formula1>
@@ -31327,6 +31330,11 @@
         <v>559</v>
       </c>
     </row>
+    <row r="185">
+      <c r="I185" s="7" t="s">
+        <v>560</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>